<commit_message>
Data driven testing (excel) update
</commit_message>
<xml_diff>
--- a/AvivaCypress/cypress/fixtures/PolicyNumbers.xlsx
+++ b/AvivaCypress/cypress/fixtures/PolicyNumbers.xlsx
@@ -406,12 +406,12 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>912501198</v>
+        <v>912501325</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>912501199</v>
+        <v>912501326</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Data driven test updates
</commit_message>
<xml_diff>
--- a/AvivaCypress/cypress/fixtures/PolicyNumbers.xlsx
+++ b/AvivaCypress/cypress/fixtures/PolicyNumbers.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -406,22 +406,47 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>912501334</v>
+        <v>912502059</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>912501336</v>
+        <v>912502060</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>912501364</v>
+        <v>912502061</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>912502062</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>912502063</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>912502064</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>912502065</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>912502066</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>